<commit_message>
Update laser manual table with new patient data: medications, HPV vaccination, smoking, comorbidities
- Added 12 new columns: MEDICATION, HPV Vaccination, Smoking Status, Cigarettes,
  Personal Medical History, Family Derm History, Immunosuppression, Wart History,
  Hyperhidrosis, Moisturizer Use, Sexual Activity, Circumcised
- Updated comorbidities for ~30 patients that had missing data
- Updated ages, treatment counts for patients with new data
- Separated medications (Verrumal, Salatac, Condylox, Gardasil 9) from past procedures
- Added 1 new patient (שמוש עזרא)
- Data merged from updated patient form (טופס מעודכן) and יבלות questionnaire

https://claude.ai/code/session_01TqAzDh5oTy45LK7B8TBozu
</commit_message>
<xml_diff>
--- a/laser final manual table.xlsx
+++ b/laser final manual table.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC113"/>
+  <dimension ref="A1:AO114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -714,6 +714,66 @@
           <t>עמודה 1</t>
         </is>
       </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>MEDICATION</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>HPV Vaccination</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Smoking Status</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Cigarettes</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>Personal Medical History</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Family Derm History</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Immunosuppression</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Wart History</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Hyperhidrosis</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Moisturizer Use</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>Sexual Activity</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Circumcised</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
@@ -836,6 +896,56 @@
         </is>
       </c>
       <c r="AC2" s="9" t="n"/>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>אם אין AD- נזלת אלרגית</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>אם אין AD- אסתמה, אם אין AD- נזלת אלרגית</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -967,6 +1077,46 @@
         </is>
       </c>
       <c r="AC3" s="9" t="n"/>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>SALATAC, VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -1094,6 +1244,46 @@
         </is>
       </c>
       <c r="AC4" s="9" t="n"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>יובש וסדקים כרוניים בכפות ידיים/רגליים</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1221,6 +1411,51 @@
         </is>
       </c>
       <c r="AC5" s="9" t="n"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>פעם ביום</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -1348,6 +1583,56 @@
         </is>
       </c>
       <c r="AC6" s="9" t="n"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -1475,6 +1760,46 @@
         </is>
       </c>
       <c r="AC7" s="9" t="n"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -1602,6 +1927,46 @@
         </is>
       </c>
       <c r="AC8" s="9" t="n"/>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>אם אין AD- אסתמה</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -1729,6 +2094,46 @@
         </is>
       </c>
       <c r="AC9" s="9" t="n"/>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>GARDASIL 9</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -1856,6 +2261,41 @@
         </is>
       </c>
       <c r="AC10" s="9" t="n"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>תרופות מדכאות חיסון</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>פעם ביום</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1983,6 +2423,46 @@
         </is>
       </c>
       <c r="AC11" s="9" t="n"/>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>BLIYABELET</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -2114,6 +2594,46 @@
         </is>
       </c>
       <c r="AC12" s="9" t="n"/>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>BLIYABELET</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>לא מעוניין.ת לענות</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -2241,6 +2761,11 @@
         </is>
       </c>
       <c r="AC13" s="9" t="n"/>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
@@ -2372,6 +2897,41 @@
         </is>
       </c>
       <c r="AC14" s="9" t="n"/>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -2499,6 +3059,41 @@
         </is>
       </c>
       <c r="AC15" s="9" t="n"/>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -2626,6 +3221,41 @@
         </is>
       </c>
       <c r="AC16" s="9" t="n"/>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -2757,6 +3387,36 @@
         </is>
       </c>
       <c r="AC17" s="9" t="n"/>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>GARDASIL 9, VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -2884,6 +3544,36 @@
         </is>
       </c>
       <c r="AC18" s="9" t="n"/>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>CONDYLOX, VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>כן, פרטנרים.ות מזדמנים.ות</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -3011,6 +3701,46 @@
         </is>
       </c>
       <c r="AC19" s="9" t="n"/>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -3138,6 +3868,46 @@
         </is>
       </c>
       <c r="AC20" s="9" t="n"/>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>CONDYLOX</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>8 כפול 6 שנים</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -3269,6 +4039,41 @@
           <t>ללא דרמוסקופיה</t>
         </is>
       </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
@@ -3394,6 +4199,51 @@
         </is>
       </c>
       <c r="AC22" s="9" t="n"/>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>GARDASIL 9, VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>כן, פרטנרים.ות מזדמנים.ות</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -3519,6 +4369,61 @@
         </is>
       </c>
       <c r="AC23" s="9" t="n"/>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס</t>
+        </is>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -3644,6 +4549,51 @@
         </is>
       </c>
       <c r="AC24" s="9" t="n"/>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>GARDASIL 9</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>כן, פרטנרים.ות מזדמנים.ות</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -3771,6 +4721,41 @@
         </is>
       </c>
       <c r="AC25" s="9" t="n"/>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>BLIYABELET</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="22.5" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
@@ -3896,6 +4881,41 @@
         </is>
       </c>
       <c r="AC26" s="9" t="n"/>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -4023,6 +5043,51 @@
         </is>
       </c>
       <c r="AC27" s="9" t="n"/>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>VERRUMAL, BLIYABELET</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס, ליכן סימפלקס</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
@@ -4148,6 +5213,41 @@
         </is>
       </c>
       <c r="AC28" s="9" t="n"/>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>UNKOWN</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>שלושה פעמים ומעלה ביום</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -4270,6 +5370,41 @@
         </is>
       </c>
       <c r="AC29" s="9" t="n"/>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
@@ -4399,6 +5534,46 @@
         </is>
       </c>
       <c r="AC30" s="9" t="n"/>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>6 כפול 1-2 שנים</t>
+        </is>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -4530,6 +5705,41 @@
         </is>
       </c>
       <c r="AC31" s="9" t="n"/>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>SALATAC, VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="22.5" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -4661,6 +5871,51 @@
         </is>
       </c>
       <c r="AC32" s="9" t="n"/>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>GARDASIL 9, CONDYLOX</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="22.5" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -4786,6 +6041,51 @@
         </is>
       </c>
       <c r="AC33" s="9" t="n"/>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>GARDASIL 9</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN33" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -4913,6 +6213,41 @@
         </is>
       </c>
       <c r="AC34" s="9" t="n"/>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="22.5" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
@@ -5040,6 +6375,41 @@
         </is>
       </c>
       <c r="AC35" s="9" t="n"/>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="22.5" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
@@ -5167,6 +6537,46 @@
         </is>
       </c>
       <c r="AC36" s="9" t="n"/>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH36" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס</t>
+        </is>
+      </c>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM36" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="22.5" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -5294,6 +6704,41 @@
         </is>
       </c>
       <c r="AC37" s="9" t="n"/>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="22.5" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
@@ -5421,6 +6866,41 @@
         </is>
       </c>
       <c r="AC38" s="9" t="n"/>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ38" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="22.5" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -5548,6 +7028,41 @@
         </is>
       </c>
       <c r="AC39" s="9" t="n"/>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="22.5" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
@@ -5675,6 +7190,46 @@
         </is>
       </c>
       <c r="AC40" s="9" t="n"/>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>7 כפול 7 שנים</t>
+        </is>
+      </c>
+      <c r="AJ40" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AN40" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="22.5" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -5802,6 +7357,51 @@
         </is>
       </c>
       <c r="AC41" s="9" t="n"/>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ41" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN41" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="AO41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="22.5" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
@@ -5929,6 +7529,56 @@
         </is>
       </c>
       <c r="AC42" s="9" t="n"/>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AI42" t="inlineStr">
+        <is>
+          <t>פסוריאזיס</t>
+        </is>
+      </c>
+      <c r="AJ42" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN42" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="22.5" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
@@ -6056,6 +7706,41 @@
         </is>
       </c>
       <c r="AC43" s="9" t="n"/>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ43" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN43" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="22.5" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
@@ -6187,6 +7872,46 @@
         </is>
       </c>
       <c r="AC44" s="9" t="n"/>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr">
+        <is>
+          <t>אם אין AD- נזלת אלרגית</t>
+        </is>
+      </c>
+      <c r="AJ44" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="22.5" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -6314,6 +8039,61 @@
         </is>
       </c>
       <c r="AC45" s="9" t="n"/>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>2 כפול 7 שנים</t>
+        </is>
+      </c>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>פסוריאזיס</t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>כן, פרטנרים.ות מזדמנים.ות</t>
+        </is>
+      </c>
+      <c r="AO45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="22.5" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -6436,6 +8216,41 @@
         </is>
       </c>
       <c r="AC46" s="9" t="n"/>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ46" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="22.5" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -6563,6 +8378,46 @@
         </is>
       </c>
       <c r="AC47" s="9" t="n"/>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>10 ביום כפול 4 שנים</t>
+        </is>
+      </c>
+      <c r="AJ47" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22.5" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
@@ -6694,6 +8549,41 @@
         </is>
       </c>
       <c r="AC48" s="9" t="n"/>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ48" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM48" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22.5" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -6821,6 +8711,51 @@
         </is>
       </c>
       <c r="AC49" s="9" t="n"/>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ49" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM49" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN49" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="22.5" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
@@ -6952,6 +8887,51 @@
         </is>
       </c>
       <c r="AC50" s="9" t="n"/>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ50" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN50" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="22.5" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
@@ -7079,6 +9059,51 @@
         </is>
       </c>
       <c r="AC51" s="9" t="n"/>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ51" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN51" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="22.5" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
@@ -7201,6 +9226,46 @@
         </is>
       </c>
       <c r="AC52" s="9" t="n"/>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ52" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="22.5" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
@@ -7328,6 +9393,46 @@
         </is>
       </c>
       <c r="AC53" s="9" t="n"/>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>VERRUMAL, SALATAC</t>
+        </is>
+      </c>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ53" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN53" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="22.5" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
@@ -7455,6 +9560,41 @@
         </is>
       </c>
       <c r="AC54" s="9" t="n"/>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ54" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="22.5" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
@@ -7582,6 +9722,41 @@
         </is>
       </c>
       <c r="AC55" s="9" t="n"/>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE55" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ55" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL55" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM55" t="inlineStr">
+        <is>
+          <t>פעם ביום</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="22.5" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
@@ -7713,6 +9888,46 @@
         </is>
       </c>
       <c r="AC56" s="9" t="n"/>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>VERRUMAL, SALATAC</t>
+        </is>
+      </c>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ56" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM56" t="inlineStr">
+        <is>
+          <t>פעם ביום</t>
+        </is>
+      </c>
+      <c r="AN56" t="inlineStr">
+        <is>
+          <t>לא מעוניין.ת לענות</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="22.5" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -7844,6 +10059,56 @@
         </is>
       </c>
       <c r="AC57" s="9" t="n"/>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>VERRUMAL, ADAFERIN</t>
+        </is>
+      </c>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH57" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס</t>
+        </is>
+      </c>
+      <c r="AJ57" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM57" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN57" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="22.5" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
@@ -7971,6 +10236,56 @@
         </is>
       </c>
       <c r="AC58" s="9" t="n"/>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AH58" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס</t>
+        </is>
+      </c>
+      <c r="AJ58" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM58" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN58" t="inlineStr">
+        <is>
+          <t>כן, פרטנרים.ות מזדמנים.ות</t>
+        </is>
+      </c>
+      <c r="AO58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="22.5" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -8102,6 +10417,46 @@
         </is>
       </c>
       <c r="AC59" s="9" t="n"/>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+      <c r="AE59" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH59" t="inlineStr">
+        <is>
+          <t>פסוריאזיס</t>
+        </is>
+      </c>
+      <c r="AJ59" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM59" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="22.5" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
@@ -8229,6 +10584,31 @@
         </is>
       </c>
       <c r="AC60" s="9" t="n"/>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AJ60" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="22.5" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
@@ -8360,6 +10740,41 @@
         </is>
       </c>
       <c r="AC61" s="9" t="n"/>
+      <c r="AD61" t="inlineStr">
+        <is>
+          <t>VERRUMAL, SALATAC</t>
+        </is>
+      </c>
+      <c r="AE61" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ61" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM61" t="inlineStr">
+        <is>
+          <t>פעם ביום</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="22.5" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
@@ -8487,6 +10902,41 @@
         </is>
       </c>
       <c r="AC62" s="9" t="n"/>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+      <c r="AE62" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ62" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM62" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="22.5" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -8614,6 +11064,46 @@
         </is>
       </c>
       <c r="AC63" s="9" t="n"/>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH63" t="inlineStr">
+        <is>
+          <t>פסוריאזיס</t>
+        </is>
+      </c>
+      <c r="AJ63" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM63" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="22.5" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
@@ -8741,10 +11231,55 @@
       </c>
       <c r="AB64" s="5" t="inlineStr">
         <is>
-          <t>PRIOR LASER</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="AC64" s="9" t="n"/>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>CONDYLOX</t>
+        </is>
+      </c>
+      <c r="AE64" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ64" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL64" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM64" t="inlineStr">
+        <is>
+          <t>פעם ביום</t>
+        </is>
+      </c>
+      <c r="AN64" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="22.5" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -8867,6 +11402,41 @@
         </is>
       </c>
       <c r="AC65" s="9" t="n"/>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>GARDASIL 9, BLIYABELT, CONDYLOX, ADAFERIN</t>
+        </is>
+      </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ65" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL65" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM65" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="22.5" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
@@ -8998,6 +11568,51 @@
         </is>
       </c>
       <c r="AC66" s="9" t="n"/>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ66" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM66" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN66" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="22.5" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -9125,6 +11740,41 @@
         </is>
       </c>
       <c r="AC67" s="9" t="n"/>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t>SALATAC, VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ67" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL67" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM67" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="22.5" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
@@ -9252,6 +11902,51 @@
         </is>
       </c>
       <c r="AC68" s="9" t="n"/>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>CONDYLOX, VERUCID</t>
+        </is>
+      </c>
+      <c r="AE68" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AJ68" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM68" t="inlineStr">
+        <is>
+          <t>לא באופן קבוע</t>
+        </is>
+      </c>
+      <c r="AN68" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="AO68" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="22.5" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
@@ -9374,6 +12069,41 @@
         </is>
       </c>
       <c r="AC69" s="9" t="n"/>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ69" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL69" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM69" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="22.5" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
@@ -9505,6 +12235,56 @@
         </is>
       </c>
       <c r="AC70" s="9" t="n"/>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH70" t="inlineStr">
+        <is>
+          <t>יובש וסדקים כרוניים בכפות ידיים/רגליים</t>
+        </is>
+      </c>
+      <c r="AJ70" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM70" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN70" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="22.5" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
@@ -9632,6 +12412,46 @@
         </is>
       </c>
       <c r="AC71" s="9" t="n"/>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH71" t="inlineStr">
+        <is>
+          <t>אם אין AD- נזלת אלרגית</t>
+        </is>
+      </c>
+      <c r="AJ71" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AN71" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="22.5" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
@@ -9759,6 +12579,11 @@
         </is>
       </c>
       <c r="AC72" s="9" t="n"/>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="22.5" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
@@ -9886,6 +12711,51 @@
         </is>
       </c>
       <c r="AC73" s="9" t="n"/>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AI73" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס</t>
+        </is>
+      </c>
+      <c r="AJ73" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM73" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN73" t="inlineStr">
+        <is>
+          <t>לא מעוניין.ת לענות</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="22.5" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
@@ -10013,6 +12883,46 @@
         </is>
       </c>
       <c r="AC74" s="9" t="n"/>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>BLIYABELT, SALATAC</t>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ74" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM74" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN74" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="22.5" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
@@ -10144,6 +13054,56 @@
         </is>
       </c>
       <c r="AC75" s="9" t="n"/>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG75" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="AJ75" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM75" t="inlineStr">
+        <is>
+          <t>לא באופן קבוע</t>
+        </is>
+      </c>
+      <c r="AN75" t="inlineStr">
+        <is>
+          <t>כן, פרטנרים.ות מזדמנים.ות</t>
+        </is>
+      </c>
+      <c r="AO75" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="22.5" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
@@ -10271,6 +13231,41 @@
         </is>
       </c>
       <c r="AC76" s="9" t="n"/>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr">
+        <is>
+          <t>Partially vaccinated</t>
+        </is>
+      </c>
+      <c r="AF76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AH76" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס, אם אין AD- אסתמה, אם אין AD- נזלת אלרגית</t>
+        </is>
+      </c>
+      <c r="AI76" t="inlineStr">
+        <is>
+          <t>אטופיק דרמטיטיס, אם אין AD- אסתמה, אם אין AD- נזלת אלרגית</t>
+        </is>
+      </c>
+      <c r="AJ76" t="inlineStr">
+        <is>
+          <t>בבירור אימונולוגי</t>
+        </is>
+      </c>
+      <c r="AK76" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="22.5" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
@@ -10402,6 +13397,46 @@
         </is>
       </c>
       <c r="AC77" s="9" t="n"/>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE77" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ77" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM77" t="inlineStr">
+        <is>
+          <t>פעם ביום</t>
+        </is>
+      </c>
+      <c r="AN77" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="22.5" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
@@ -10529,6 +13564,51 @@
         </is>
       </c>
       <c r="AC78" s="9" t="n"/>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
+          <t>Fully vaccinated</t>
+        </is>
+      </c>
+      <c r="AF78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ78" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM78" t="inlineStr">
+        <is>
+          <t>כמה פעמים בשבוע</t>
+        </is>
+      </c>
+      <c r="AN78" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="22.5" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
@@ -10658,6 +13738,51 @@
         </is>
       </c>
       <c r="AC79" s="9" t="n"/>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>SALATAC, VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ79" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AM79" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN79" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO79" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="22.5" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
@@ -10787,6 +13912,51 @@
         </is>
       </c>
       <c r="AC80" s="9" t="n"/>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AJ80" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM80" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN80" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO80" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="22.5" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
@@ -10913,6 +14083,51 @@
         </is>
       </c>
       <c r="AC81" s="9" t="n"/>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AE81" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AJ81" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK81" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AL81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM81" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN81" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+      <c r="AO81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="22.5" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
@@ -11038,6 +14253,56 @@
         </is>
       </c>
       <c r="AC82" s="9" t="n"/>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AE82" t="inlineStr">
+        <is>
+          <t>Not vaccinated</t>
+        </is>
+      </c>
+      <c r="AF82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG82" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="AJ82" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="AK82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AL82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AM82" t="inlineStr">
+        <is>
+          <t>לא משתמש.ת בכלל</t>
+        </is>
+      </c>
+      <c r="AN82" t="inlineStr">
+        <is>
+          <t>כן, פרטנר.ית קבוע.ה</t>
+        </is>
+      </c>
+      <c r="AO82" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="22.5" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
@@ -11165,6 +14430,21 @@
         </is>
       </c>
       <c r="AC83" s="9" t="n"/>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
+      <c r="AF83" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AJ83" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="22.5" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -11281,7 +14561,7 @@
       </c>
       <c r="Y84" s="5" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>mycosis funoidosis</t>
         </is>
       </c>
       <c r="Z84" s="8" t="n">
@@ -11296,6 +14576,11 @@
         </is>
       </c>
       <c r="AC84" s="9" t="n"/>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="22.5" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
@@ -11427,6 +14712,11 @@
         </is>
       </c>
       <c r="AC85" s="9" t="n"/>
+      <c r="AD85" t="inlineStr">
+        <is>
+          <t>SALATAC, VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="22.5" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
@@ -11558,6 +14848,11 @@
         </is>
       </c>
       <c r="AC86" s="9" t="n"/>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>CONDYLOX, VERUCID</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="22.5" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -11573,7 +14868,9 @@
           <t>052-8138433</t>
         </is>
       </c>
-      <c r="D87" s="5" t="n"/>
+      <c r="D87" s="5" t="n">
+        <v>46</v>
+      </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -11665,7 +14962,11 @@
           <t>healed</t>
         </is>
       </c>
-      <c r="Y87" s="5" t="n"/>
+      <c r="Y87" s="5" t="inlineStr">
+        <is>
+          <t>METABOLIC DIS</t>
+        </is>
+      </c>
       <c r="Z87" s="8" t="n">
         <v>45949</v>
       </c>
@@ -11678,6 +14979,11 @@
         </is>
       </c>
       <c r="AC87" s="9" t="n"/>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="22.5" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
@@ -11693,7 +14999,9 @@
           <t>054-4246255</t>
         </is>
       </c>
-      <c r="D88" s="5" t="n"/>
+      <c r="D88" s="5" t="n">
+        <v>23</v>
+      </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -11705,7 +15013,7 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
@@ -11790,7 +15098,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y88" s="5" t="n"/>
+      <c r="Y88" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z88" s="8" t="n">
         <v>46009</v>
       </c>
@@ -11803,6 +15115,11 @@
         </is>
       </c>
       <c r="AC88" s="9" t="n"/>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>BLIYABELET</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="22.5" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -11818,7 +15135,9 @@
           <t>052-3260747</t>
         </is>
       </c>
-      <c r="D89" s="5" t="n"/>
+      <c r="D89" s="5" t="n">
+        <v>68.2</v>
+      </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -11830,7 +15149,7 @@
         </is>
       </c>
       <c r="G89" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H89" s="7" t="n"/>
       <c r="I89" s="7" t="inlineStr">
@@ -11911,7 +15230,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y89" s="5" t="n"/>
+      <c r="Y89" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z89" s="8" t="n">
         <v>46000</v>
       </c>
@@ -11920,10 +15243,15 @@
       </c>
       <c r="AB89" s="5" t="inlineStr">
         <is>
-          <t>treatment unspecified</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="AC89" s="9" t="n"/>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="22.5" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
@@ -12034,7 +15362,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y90" s="5" t="n"/>
+      <c r="Y90" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z90" s="8" t="n">
         <v>45997</v>
       </c>
@@ -12047,6 +15379,11 @@
         </is>
       </c>
       <c r="AC90" s="9" t="n"/>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="22.5" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
@@ -12062,7 +15399,9 @@
           <t>052-3600098</t>
         </is>
       </c>
-      <c r="D91" s="5" t="n"/>
+      <c r="D91" s="5" t="n">
+        <v>16</v>
+      </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -12073,7 +15412,9 @@
           <t>רגליים (לא כפות)</t>
         </is>
       </c>
-      <c r="G91" s="4" t="n"/>
+      <c r="G91" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="H91" s="7" t="n"/>
       <c r="I91" s="7" t="inlineStr">
         <is>
@@ -12153,7 +15494,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y91" s="5" t="n"/>
+      <c r="Y91" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z91" s="8" t="n">
         <v>45938</v>
       </c>
@@ -12166,6 +15511,11 @@
         </is>
       </c>
       <c r="AC91" s="9" t="n"/>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>BLIYABELET</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="22.5" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
@@ -12181,7 +15531,9 @@
           <t>054-5753520</t>
         </is>
       </c>
-      <c r="D92" s="5" t="n"/>
+      <c r="D92" s="5" t="n">
+        <v>38</v>
+      </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -12278,7 +15630,11 @@
           <t>healed</t>
         </is>
       </c>
-      <c r="Y92" s="5" t="n"/>
+      <c r="Y92" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z92" s="8" t="n">
         <v>45945</v>
       </c>
@@ -12287,10 +15643,15 @@
       </c>
       <c r="AB92" s="5" t="inlineStr">
         <is>
-          <t>Solution</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="AC92" s="9" t="n"/>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>CONDYLOX, GARDASIL 9</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="22.5" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
@@ -12306,7 +15667,9 @@
           <t>054-2957195</t>
         </is>
       </c>
-      <c r="D93" s="5" t="n"/>
+      <c r="D93" s="5" t="n">
+        <v>18</v>
+      </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -12318,7 +15681,7 @@
         </is>
       </c>
       <c r="G93" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H93" s="7" t="n"/>
       <c r="I93" s="7" t="inlineStr">
@@ -12399,7 +15762,11 @@
           <t>no answer</t>
         </is>
       </c>
-      <c r="Y93" s="5" t="n"/>
+      <c r="Y93" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z93" s="8" t="n">
         <v>46043</v>
       </c>
@@ -12412,6 +15779,11 @@
         </is>
       </c>
       <c r="AC93" s="9" t="n"/>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="22.5" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
@@ -12427,7 +15799,9 @@
           <t>054-7588625</t>
         </is>
       </c>
-      <c r="D94" s="5" t="n"/>
+      <c r="D94" s="5" t="n">
+        <v>50</v>
+      </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -12516,7 +15890,11 @@
           <t>healed</t>
         </is>
       </c>
-      <c r="Y94" s="5" t="n"/>
+      <c r="Y94" s="5" t="inlineStr">
+        <is>
+          <t>SMOKING</t>
+        </is>
+      </c>
       <c r="Z94" s="8" t="n">
         <v>46049</v>
       </c>
@@ -12525,10 +15903,15 @@
       </c>
       <c r="AB94" s="5" t="inlineStr">
         <is>
-          <t>EC, Liquid Nitrogen</t>
+          <t>Liquid Nitrogen, EC</t>
         </is>
       </c>
       <c r="AC94" s="9" t="n"/>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>CONDYLOX</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="22.5" customHeight="1">
       <c r="A95" s="4" t="inlineStr">
@@ -12544,7 +15927,9 @@
           <t>054-5780440</t>
         </is>
       </c>
-      <c r="D95" s="5" t="n"/>
+      <c r="D95" s="5" t="n">
+        <v>26.11</v>
+      </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
           <t>זכר</t>
@@ -12556,7 +15941,7 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H95" s="7" t="inlineStr">
         <is>
@@ -12637,7 +16022,11 @@
           <t>healed</t>
         </is>
       </c>
-      <c r="Y95" s="5" t="n"/>
+      <c r="Y95" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z95" s="8" t="n">
         <v>45652</v>
       </c>
@@ -12646,10 +16035,15 @@
       </c>
       <c r="AB95" s="5" t="inlineStr">
         <is>
-          <t>EC, Liquid Nitrogen, Verrumal</t>
+          <t>Liquid Nitrogen, EC</t>
         </is>
       </c>
       <c r="AC95" s="9" t="n"/>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>GARDASIL 9, VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="22.5" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
@@ -12665,7 +16059,9 @@
           <t>050-9496143</t>
         </is>
       </c>
-      <c r="D96" s="5" t="n"/>
+      <c r="D96" s="5" t="n">
+        <v>23.5</v>
+      </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
           <t>נקבה</t>
@@ -12758,7 +16154,11 @@
           <t>healed</t>
         </is>
       </c>
-      <c r="Y96" s="5" t="n"/>
+      <c r="Y96" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z96" s="8" t="n">
         <v>46016</v>
       </c>
@@ -12767,10 +16167,15 @@
       </c>
       <c r="AB96" s="5" t="inlineStr">
         <is>
-          <t>Bliyabelet</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="AC96" s="9" t="n"/>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>BLIYABELET</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="22.5" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
@@ -12800,7 +16205,7 @@
         </is>
       </c>
       <c r="G97" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
@@ -12898,10 +16303,15 @@
       </c>
       <c r="AB97" s="5" t="inlineStr">
         <is>
-          <t>Prior Bx</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="AC97" s="9" t="n"/>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="22.5" customHeight="1">
       <c r="A98" s="4" t="inlineStr">
@@ -13029,6 +16439,11 @@
         </is>
       </c>
       <c r="AC98" s="9" t="n"/>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>GARDASIL 9</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="22.5" customHeight="1">
       <c r="A99" s="4" t="inlineStr">
@@ -13156,6 +16571,11 @@
         </is>
       </c>
       <c r="AC99" s="9" t="n"/>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="22.5" customHeight="1">
       <c r="A100" s="4" t="inlineStr">
@@ -13261,7 +16681,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y100" s="5" t="n"/>
+      <c r="Y100" s="5" t="inlineStr">
+        <is>
+          <t>HYPERTENSION</t>
+        </is>
+      </c>
       <c r="Z100" s="8" t="n">
         <v>45993</v>
       </c>
@@ -13274,6 +16698,11 @@
         </is>
       </c>
       <c r="AC100" s="9" t="n"/>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="22.5" customHeight="1">
       <c r="A101" s="4" t="inlineStr">
@@ -13303,7 +16732,7 @@
         </is>
       </c>
       <c r="G101" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H101" s="7" t="n"/>
       <c r="I101" s="7" t="n"/>
@@ -13375,7 +16804,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y101" s="5" t="n"/>
+      <c r="Y101" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z101" s="8" t="n">
         <v>46051</v>
       </c>
@@ -13384,10 +16817,15 @@
       </c>
       <c r="AB101" s="5" t="inlineStr">
         <is>
-          <t>Liquid Nitrogen</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="AC101" s="9" t="n"/>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="22.5" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
@@ -13417,7 +16855,7 @@
         </is>
       </c>
       <c r="G102" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H102" s="7" t="inlineStr">
         <is>
@@ -13502,7 +16940,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y102" s="5" t="n"/>
+      <c r="Y102" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z102" s="8" t="n">
         <v>45777</v>
       </c>
@@ -13511,10 +16953,15 @@
       </c>
       <c r="AB102" s="5" t="inlineStr">
         <is>
-          <t>Liquid Nitrogen, SALATAC</t>
+          <t>Liquid Nitrogen</t>
         </is>
       </c>
       <c r="AC102" s="9" t="n"/>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t>SALATAC, VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="22.5" customHeight="1">
       <c r="A103" s="4" t="inlineStr">
@@ -13625,7 +17072,11 @@
           <t>healed</t>
         </is>
       </c>
-      <c r="Y103" s="5" t="n"/>
+      <c r="Y103" s="5" t="inlineStr">
+        <is>
+          <t>SKIN MALIGNANCY</t>
+        </is>
+      </c>
       <c r="Z103" s="8" t="n">
         <v>46064</v>
       </c>
@@ -13634,10 +17085,15 @@
       </c>
       <c r="AB103" s="5" t="inlineStr">
         <is>
+          <t>Liquid Nitrogen</t>
+        </is>
+      </c>
+      <c r="AC103" s="9" t="n"/>
+      <c r="AD103" t="inlineStr">
+        <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="AC103" s="9" t="n"/>
     </row>
     <row r="104" ht="22.5" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
@@ -13667,7 +17123,7 @@
         </is>
       </c>
       <c r="G104" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H104" s="7" t="n"/>
       <c r="I104" s="7" t="inlineStr">
@@ -13748,7 +17204,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y104" s="5" t="n"/>
+      <c r="Y104" s="5" t="inlineStr">
+        <is>
+          <t>METABOLIC DIS, SMOKING</t>
+        </is>
+      </c>
       <c r="Z104" s="8" t="n">
         <v>45997</v>
       </c>
@@ -13761,6 +17221,11 @@
         </is>
       </c>
       <c r="AC104" s="9" t="n"/>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>GARDASIL 9</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="22.5" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
@@ -13875,7 +17340,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y105" s="5" t="n"/>
+      <c r="Y105" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z105" s="8" t="n">
         <v>45720</v>
       </c>
@@ -13884,10 +17353,15 @@
       </c>
       <c r="AB105" s="5" t="inlineStr">
         <is>
-          <t>Liquid Nitrogen, Verrumal</t>
+          <t>Liquid Nitrogen</t>
         </is>
       </c>
       <c r="AC105" s="9" t="n"/>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="22.5" customHeight="1">
       <c r="A106" s="4" t="inlineStr">
@@ -13998,7 +17472,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y106" s="5" t="n"/>
+      <c r="Y106" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z106" s="8" t="n">
         <v>46065</v>
       </c>
@@ -14007,10 +17485,15 @@
       </c>
       <c r="AB106" s="5" t="inlineStr">
         <is>
-          <t>Liquid Nitrogen, EC</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="AC106" s="9" t="n"/>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="22.5" customHeight="1">
       <c r="A107" s="4" t="inlineStr">
@@ -14121,7 +17604,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y107" s="5" t="n"/>
+      <c r="Y107" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z107" s="8" t="n">
         <v>46065</v>
       </c>
@@ -14130,10 +17617,15 @@
       </c>
       <c r="AB107" s="5" t="inlineStr">
         <is>
-          <t>Liquid Nitrogen, Verrumal</t>
+          <t>Liquid Nitrogen</t>
         </is>
       </c>
       <c r="AC107" s="9" t="n"/>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>VERRUMAL, VERUCID</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="22.5" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
@@ -14248,7 +17740,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y108" s="5" t="n"/>
+      <c r="Y108" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z108" s="8" t="n">
         <v>45949</v>
       </c>
@@ -14257,10 +17753,15 @@
       </c>
       <c r="AB108" s="5" t="inlineStr">
         <is>
-          <t>Verrumal</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="AC108" s="9" t="n"/>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>SALATAC, VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="22.5" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
@@ -14371,7 +17872,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y109" s="5" t="n"/>
+      <c r="Y109" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z109" s="8" t="n">
         <v>46078</v>
       </c>
@@ -14384,6 +17889,11 @@
         </is>
       </c>
       <c r="AC109" s="9" t="n"/>
+      <c r="AD109" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="22.5" customHeight="1">
       <c r="A110" s="4" t="inlineStr">
@@ -14498,7 +18008,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y110" s="5" t="n"/>
+      <c r="Y110" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z110" s="8" t="n">
         <v>45928</v>
       </c>
@@ -14507,10 +18021,15 @@
       </c>
       <c r="AB110" s="5" t="inlineStr">
         <is>
-          <t>Verrumal, Condylox</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="AC110" s="9" t="n"/>
+      <c r="AD110" t="inlineStr">
+        <is>
+          <t>CONDYLOX, VERRUMAL</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="22.5" customHeight="1">
       <c r="A111" s="4" t="inlineStr">
@@ -14621,7 +18140,11 @@
           <t>healed</t>
         </is>
       </c>
-      <c r="Y111" s="5" t="n"/>
+      <c r="Y111" s="5" t="inlineStr">
+        <is>
+          <t>SMOKING</t>
+        </is>
+      </c>
       <c r="Z111" s="8" t="n">
         <v>46089</v>
       </c>
@@ -14632,6 +18155,11 @@
         </is>
       </c>
       <c r="AC111" s="9" t="n"/>
+      <c r="AD111" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="22.5" customHeight="1">
       <c r="A112" s="11" t="inlineStr">
@@ -14661,7 +18189,7 @@
         </is>
       </c>
       <c r="G112" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H112" s="7" t="n"/>
       <c r="I112" s="7" t="inlineStr">
@@ -14742,7 +18270,11 @@
           <t>not healed</t>
         </is>
       </c>
-      <c r="Y112" s="5" t="n"/>
+      <c r="Y112" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
       <c r="Z112" s="8" t="n">
         <v>46089</v>
       </c>
@@ -14755,6 +18287,11 @@
         </is>
       </c>
       <c r="AC112" s="9" t="n"/>
+      <c r="AD112" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="22.5" customHeight="1">
       <c r="A113" t="inlineStr">
@@ -14784,7 +18321,7 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
@@ -14869,6 +18406,11 @@
           <t>healed</t>
         </is>
       </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>AUTO IMMUNE</t>
+        </is>
+      </c>
       <c r="Z113" s="21" t="n">
         <v>45973</v>
       </c>
@@ -14877,7 +18419,73 @@
       </c>
       <c r="AB113" t="inlineStr">
         <is>
-          <t>Liquid Nitrogen, EC, SALATAC</t>
+          <t>Liquid Nitrogen, EC, Solution</t>
+        </is>
+      </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t>SALATAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>שמוש עזרא</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>55648117</v>
+      </c>
+      <c r="D114" t="n">
+        <v>67</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>זכר</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>גב</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>3</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2-400, 500 PIXEL</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>2940nm only</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>METABOLIC DIS, SKIN MALIGNANCY</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>2025-10-19</t>
+        </is>
+      </c>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>2025-01-06</t>
+        </is>
+      </c>
+      <c r="AB114" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t>NONE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore 2 excluded patients (N=105→107): assign both to Nd:YAG 1064nm group
Treatment group identified from clinical records:
- צדי מור חיים (ID 38440244): LP Nd:YAG, condylomata, healed
- שמואלי אסף (ID 339999195): LP Nd:YAG 160J/2mm + 50J/6mm, palmoplantar, not healed

Key statistical changes:
- Frog-spawn: p=0.118 → p=0.046 (now significant, Chi²)
- Condylomata frog-spawn: OR=0.23, p=0.050 → OR=0.18, p=0.022
- 1064nm group: 48→50 patients, clearance 54.2%→54.0%
- MV HK grade: OR=2.43, p=0.028 → OR=2.07, p=0.107 (now trend)
- MV frog-spawn: OR=0.65, p=0.411 → OR=0.39, p=0.152
- CV AUC: 0.778 → 0.776

https://claude.ai/code/session_01TqAzDh5oTy45LK7B8TBozu
</commit_message>
<xml_diff>
--- a/laser final manual table.xlsx
+++ b/laser final manual table.xlsx
@@ -15815,11 +15815,13 @@
       <c r="G94" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H94" s="7" t="n"/>
+      <c r="H94" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I94" s="7" t="n"/>
       <c r="J94" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1064nm only</t>
         </is>
       </c>
       <c r="K94" s="5" t="inlineStr">
@@ -16734,11 +16736,13 @@
       <c r="G101" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H101" s="7" t="n"/>
+      <c r="H101" s="7" t="n">
+        <v>3</v>
+      </c>
       <c r="I101" s="7" t="n"/>
       <c r="J101" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1064nm only</t>
         </is>
       </c>
       <c r="K101" s="5" t="inlineStr">

</xml_diff>